<commit_message>
Remove test serial records
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1244"/>
+  <dimension ref="A1:E1243"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -21552,26 +21552,9 @@
         <v/>
       </c>
     </row>
-    <row r="1244">
-      <c r="A1244" t="str">
-        <v>99995</v>
-      </c>
-      <c r="B1244" t="str">
-        <v>СТАНДАРТ</v>
-      </c>
-      <c r="C1244" t="str">
-        <v>08.06.2026</v>
-      </c>
-      <c r="D1244" t="str">
-        <v/>
-      </c>
-      <c r="E1244" t="str">
-        <v>2026-06-08T18:05:03.590Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1244"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1243"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>